<commit_message>
NT track diff Vanguard EU update
</commit_message>
<xml_diff>
--- a/NorthernTrust/NT-KostenBepaling.xlsx
+++ b/NorthernTrust/NT-KostenBepaling.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c741cee80ec8cf3/Financieel/IndexFondsenOnderzoek/KeuzeWelkIndexFonds/OnderzoekPerFonds/NorthernTrust/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="750" documentId="13_ncr:1_{0BEEB54A-A1B5-4808-9253-8C962E6DCC11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3B76FBF-B5DA-43D1-BE16-84A1CFEFB23C}"/>
+  <xr:revisionPtr revIDLastSave="770" documentId="13_ncr:1_{0BEEB54A-A1B5-4808-9253-8C962E6DCC11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{757603FA-61CE-45CD-B00D-0ACBF722F1CE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aannames" sheetId="4" r:id="rId1"/>
@@ -5022,8 +5022,8 @@
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
       <c r="P6" s="19">
-        <f>AVERAGE(E6:L6)</f>
-        <v>0.34999999999999937</v>
+        <f>AVERAGE(E6:M6)</f>
+        <v>0.32444444444444359</v>
       </c>
     </row>
     <row r="7" spans="2:36" x14ac:dyDescent="0.25">
@@ -5099,9 +5099,15 @@
       <c r="J10" s="22">
         <v>3.81</v>
       </c>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
+      <c r="K10" s="22">
+        <v>-15.57</v>
+      </c>
+      <c r="L10" s="22">
+        <v>5.57</v>
+      </c>
+      <c r="M10" s="22">
+        <v>15.02</v>
+      </c>
       <c r="N10" s="22"/>
       <c r="O10" s="20"/>
       <c r="P10" s="22"/>
@@ -5165,9 +5171,15 @@
       <c r="J12" s="22">
         <v>3.74</v>
       </c>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="22"/>
+      <c r="K12" s="22">
+        <v>-15.59</v>
+      </c>
+      <c r="L12" s="22">
+        <v>5.89</v>
+      </c>
+      <c r="M12" s="22">
+        <v>14.95</v>
+      </c>
       <c r="N12" s="22"/>
       <c r="O12" s="20"/>
       <c r="P12" s="22"/>
@@ -5179,7 +5191,7 @@
       <c r="C13" s="22"/>
       <c r="D13" s="22"/>
       <c r="E13" s="22">
-        <f t="shared" ref="E13:J13" si="2">E10-E12</f>
+        <f t="shared" ref="E13:M13" si="2">E10-E12</f>
         <v>-0.20000000000000107</v>
       </c>
       <c r="F13" s="22">
@@ -5202,14 +5214,23 @@
         <f t="shared" si="2"/>
         <v>6.999999999999984E-2</v>
       </c>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22"/>
-      <c r="M13" s="22"/>
+      <c r="K13" s="22">
+        <f t="shared" si="2"/>
+        <v>1.9999999999999574E-2</v>
+      </c>
+      <c r="L13" s="22">
+        <f t="shared" si="2"/>
+        <v>-0.3199999999999994</v>
+      </c>
+      <c r="M13" s="22">
+        <f t="shared" si="2"/>
+        <v>7.0000000000000284E-2</v>
+      </c>
       <c r="N13" s="22"/>
       <c r="O13" s="22"/>
       <c r="P13" s="22">
-        <f>AVERAGE(E13:J13)</f>
-        <v>2.4999999999999689E-2</v>
+        <f>AVERAGE(E13:M13)</f>
+        <v>-8.888888888889045E-3</v>
       </c>
       <c r="AB13" s="1">
         <f t="shared" ref="AB13:AD13" si="3">E2</f>
@@ -5224,7 +5245,7 @@
         <v>2018</v>
       </c>
       <c r="AE13" s="1">
-        <f t="shared" ref="AE13:AJ15" si="4">H2</f>
+        <f t="shared" ref="AE13:AJ14" si="4">H2</f>
         <v>2019</v>
       </c>
       <c r="AF13" s="1">
@@ -5283,7 +5304,7 @@
       <c r="M14" s="22"/>
       <c r="N14" s="22"/>
       <c r="O14" s="27">
-        <f>AVERAGE(E14:J14)</f>
+        <f>AVERAGE(E14:M14)</f>
         <v>0.36500000000000027</v>
       </c>
       <c r="P14" s="22"/>
@@ -5332,39 +5353,39 @@
         <v>123</v>
       </c>
       <c r="AB16" s="26">
-        <f>AB20-AB14</f>
+        <f t="shared" ref="AB16:AJ16" si="7">AB20-AB14</f>
         <v>0.16999999999999993</v>
       </c>
       <c r="AC16" s="26">
-        <f>AC20-AC14</f>
+        <f t="shared" si="7"/>
         <v>0.21999999999999886</v>
       </c>
       <c r="AD16" s="26">
-        <f>AD20-AD14</f>
+        <f t="shared" si="7"/>
         <v>0.17999999999999972</v>
       </c>
       <c r="AE16" s="26">
-        <f>AE20-AE14</f>
+        <f t="shared" si="7"/>
         <v>0.24000000000000199</v>
       </c>
       <c r="AF16" s="26">
-        <f>AF20-AF14</f>
+        <f t="shared" si="7"/>
         <v>0.30999999999999872</v>
       </c>
       <c r="AG16" s="26">
-        <f>AG20-AG14</f>
+        <f t="shared" si="7"/>
         <v>0.25</v>
       </c>
       <c r="AH16" s="26">
-        <f>AH20-AH14</f>
+        <f t="shared" si="7"/>
         <v>0.12000000000000099</v>
       </c>
       <c r="AI16" s="26">
-        <f>AI20-AI14</f>
+        <f t="shared" si="7"/>
         <v>0.34999999999999787</v>
       </c>
       <c r="AJ16" s="26">
-        <f>AJ20-AJ14</f>
+        <f t="shared" si="7"/>
         <v>0.42999999999999972</v>
       </c>
     </row>
@@ -5497,15 +5518,15 @@
         <v>0.71999999999999886</v>
       </c>
       <c r="F20">
-        <f t="shared" ref="F20:H20" si="7">F19-F18</f>
+        <f t="shared" ref="F20:H20" si="8">F19-F18</f>
         <v>0.62000000000000011</v>
       </c>
       <c r="G20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.55999999999999994</v>
       </c>
       <c r="H20">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.77999999999999403</v>
       </c>
       <c r="N20">
@@ -5516,39 +5537,39 @@
         <v>122</v>
       </c>
       <c r="AB20" s="26">
-        <f>E4</f>
+        <f t="shared" ref="AB20:AJ20" si="9">E4</f>
         <v>10.72</v>
       </c>
       <c r="AC20" s="26">
-        <f>F4</f>
+        <f t="shared" si="9"/>
         <v>8.5399999999999991</v>
       </c>
       <c r="AD20" s="26">
-        <f>G4</f>
+        <f t="shared" si="9"/>
         <v>-3.12</v>
       </c>
       <c r="AE20" s="26">
-        <f>H4</f>
+        <f t="shared" si="9"/>
         <v>31.17</v>
       </c>
       <c r="AF20" s="26">
-        <f>I4</f>
+        <f t="shared" si="9"/>
         <v>8.5299999999999994</v>
       </c>
       <c r="AG20" s="26">
-        <f>J4</f>
+        <f t="shared" si="9"/>
         <v>31.99</v>
       </c>
       <c r="AH20" s="26">
-        <f>K4</f>
+        <f t="shared" si="9"/>
         <v>-13.59</v>
       </c>
       <c r="AI20" s="26">
-        <f>L4</f>
+        <f t="shared" si="9"/>
         <v>20.86</v>
       </c>
       <c r="AJ20" s="26">
-        <f>M4</f>
+        <f t="shared" si="9"/>
         <v>27.4</v>
       </c>
     </row>
@@ -5561,15 +5582,15 @@
         <v>0.27999999999999936</v>
       </c>
       <c r="F21">
-        <f t="shared" ref="F21:H21" si="8">F17-F18</f>
+        <f t="shared" ref="F21:H21" si="10">F17-F18</f>
         <v>0.30000000000000071</v>
       </c>
       <c r="G21">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.32999999999999996</v>
       </c>
       <c r="H21">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0.45999999999999375</v>
       </c>
       <c r="P21" s="26">
@@ -5580,39 +5601,39 @@
         <v>126</v>
       </c>
       <c r="AB21" s="26">
-        <f>AB16-AB17</f>
+        <f t="shared" ref="AB21:AJ21" si="11">AB16-AB17</f>
         <v>0.13999999999999993</v>
       </c>
       <c r="AC21" s="26">
-        <f>AC16-AC17</f>
+        <f t="shared" si="11"/>
         <v>0.18999999999999886</v>
       </c>
       <c r="AD21" s="26">
-        <f>AD16-AD17</f>
+        <f t="shared" si="11"/>
         <v>5.999999999999972E-2</v>
       </c>
       <c r="AE21" s="26">
-        <f>AE16-AE17</f>
+        <f t="shared" si="11"/>
         <v>9.0000000000001995E-2</v>
       </c>
       <c r="AF21" s="26">
-        <f>AF16-AF17</f>
+        <f t="shared" si="11"/>
         <v>0.15999999999999873</v>
       </c>
       <c r="AG21" s="26">
-        <f>AG16-AG17</f>
+        <f t="shared" si="11"/>
         <v>0.1</v>
       </c>
       <c r="AH21" s="26">
-        <f>AH16-AH17</f>
+        <f t="shared" si="11"/>
         <v>-2.9999999999999E-2</v>
       </c>
       <c r="AI21" s="26">
-        <f>AI16-AI17</f>
+        <f t="shared" si="11"/>
         <v>0.19999999999999787</v>
       </c>
       <c r="AJ21" s="26">
-        <f>AJ16-AJ17</f>
+        <f t="shared" si="11"/>
         <v>0.27999999999999969</v>
       </c>
     </row>
@@ -5625,15 +5646,15 @@
         <v>0.4399999999999995</v>
       </c>
       <c r="F22">
-        <f t="shared" ref="F22:H22" si="9">F19-F17</f>
+        <f t="shared" ref="F22:H22" si="12">F19-F17</f>
         <v>0.3199999999999994</v>
       </c>
       <c r="G22">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0.22999999999999998</v>
       </c>
       <c r="H22">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0.32000000000000028</v>
       </c>
       <c r="O22" s="28">
@@ -5701,15 +5722,15 @@
         <v>0.65999999999999992</v>
       </c>
       <c r="F28">
-        <f t="shared" ref="F28:H28" si="10">F27-F26</f>
+        <f t="shared" ref="F28:H28" si="13">F27-F26</f>
         <v>0.66000000000000014</v>
       </c>
       <c r="G28">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.58999999999999986</v>
       </c>
       <c r="H28">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>0.84999999999999787</v>
       </c>
       <c r="N28">
@@ -5726,15 +5747,15 @@
         <v>0.57000000000000006</v>
       </c>
       <c r="F29">
-        <f t="shared" ref="F29:H29" si="11">F25-F26</f>
+        <f t="shared" ref="F29:H29" si="14">F25-F26</f>
         <v>0.48999999999999844</v>
       </c>
       <c r="G29">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.41999999999999993</v>
       </c>
       <c r="H29">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.62000000000000099</v>
       </c>
       <c r="P29" s="26">
@@ -5751,15 +5772,15 @@
         <v>8.9999999999999858E-2</v>
       </c>
       <c r="F30">
-        <f t="shared" ref="F30:H30" si="12">F27-F25</f>
+        <f t="shared" ref="F30:H30" si="15">F27-F25</f>
         <v>0.17000000000000171</v>
       </c>
       <c r="G30">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.16999999999999993</v>
       </c>
       <c r="H30">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.22999999999999687</v>
       </c>
       <c r="O30" s="28">
@@ -5777,6 +5798,15 @@
       <c r="J33">
         <v>23.91</v>
       </c>
+      <c r="K33">
+        <v>-15.2</v>
+      </c>
+      <c r="L33">
+        <v>12.01</v>
+      </c>
+      <c r="M33">
+        <v>14.23</v>
+      </c>
     </row>
     <row r="34" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B34" s="21" t="s">
@@ -5799,6 +5829,15 @@
       <c r="J35">
         <v>23.9</v>
       </c>
+      <c r="K35">
+        <v>-15.41</v>
+      </c>
+      <c r="L35">
+        <v>11.86</v>
+      </c>
+      <c r="M35">
+        <v>14.11</v>
+      </c>
     </row>
     <row r="36" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B36" s="21" t="s">
@@ -5812,9 +5851,21 @@
         <f>J33-J35</f>
         <v>1.0000000000001563E-2</v>
       </c>
+      <c r="K36">
+        <f t="shared" ref="K36:M36" si="16">K33-K35</f>
+        <v>0.21000000000000085</v>
+      </c>
+      <c r="L36">
+        <f t="shared" si="16"/>
+        <v>0.15000000000000036</v>
+      </c>
+      <c r="M36">
+        <f t="shared" si="16"/>
+        <v>0.12000000000000099</v>
+      </c>
       <c r="P36" s="26">
-        <f>AVERAGE(I36:J36)</f>
-        <v>8.5000000000000853E-2</v>
+        <f>AVERAGE(I36:M36)</f>
+        <v>0.13000000000000078</v>
       </c>
     </row>
     <row r="37" spans="2:16" x14ac:dyDescent="0.25">
@@ -5830,7 +5881,7 @@
         <v>0.44000000000000128</v>
       </c>
       <c r="O37" s="29">
-        <f>AVERAGE(I37:J37)</f>
+        <f>AVERAGE(I37:M37)</f>
         <v>0.36500000000000021</v>
       </c>
     </row>
@@ -5922,8 +5973,8 @@
       <c r="B63" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="AB20:AJ20">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="AB19:AJ19">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -5934,8 +5985,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB19:AJ19">
-    <cfRule type="colorScale" priority="3">
+  <conditionalFormatting sqref="AB20:AJ20">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>